<commit_message>
v2/v3: correcoes de engenharia, P95 segmentado, novas camadas analiticas e PT-BR
- Notebooks v2 (pipeline + analise) e v3 (analise):
  - Caminhos via pathlib; fim da fragmentacao de DataFrame; warnings direcionados; fallback de fonte.
  - Graficos redesenhados (data storytelling); meses em PT-BR (sem locale), acentuacao e graus Celsius.
  - P95 automatizado e SEGMENTADO por UHE (BM=ETE01+02; PM=ETE PM+Compacta), com rastreabilidade.
- v3: 4 camadas novas -> pos-hoc de Dunn (scikit-posthocs), deteccao de ruptura (ruptures),
  validacao de schema (pandera) e outliers por IQR. Relatorio mestre v3 multi-aba.
- VMPs marcados como "conferir na base" (nao validados automaticamente).
- README reescrito (historico de versoes, camadas v3, nota regulatoria, execucao headless).
- Adicionado .gitignore (.ipynb_checkpoints, auxiliares de build).
- Produtos (PNGs e planilhas) regenerados.
</commit_message>
<xml_diff>
--- a/produtos/Relatorio_Diluicao_Mestre_Segregado.xlsx
+++ b/produtos/Relatorio_Diluicao_Mestre_Segregado.xlsx
@@ -16,7 +16,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
   <si>
-    <t>Mês/Ano</t>
+    <t>Mes/Ano</t>
   </si>
   <si>
     <t>Q_BeloMonte_m3s</t>
@@ -564,13 +564,13 @@
         <v>4361597.642536836</v>
       </c>
       <c r="F2">
-        <v>2.035492662921628E-05</v>
+        <v>1.974505836120868E-05</v>
       </c>
       <c r="G2">
-        <v>1.031732032343695E-05</v>
+        <v>6.099829049000893E-05</v>
       </c>
       <c r="H2">
-        <v>1.031732032343695E-06</v>
+        <v>2.017609307694338E-06</v>
       </c>
       <c r="I2">
         <v>1103</v>
@@ -585,13 +585,13 @@
         <v>26662754.11764706</v>
       </c>
       <c r="M2">
-        <v>3.329738541197434E-06</v>
+        <v>7.064911567981084E-06</v>
       </c>
       <c r="N2">
-        <v>1.687747627324674E-06</v>
+        <v>6.907013401069154E-06</v>
       </c>
       <c r="O2">
-        <v>1.687747627324674E-07</v>
+        <v>1.043778143743237E-06</v>
       </c>
     </row>
     <row r="3" spans="1:15">
@@ -611,13 +611,13 @@
         <v>16417208.76636802</v>
       </c>
       <c r="F3">
-        <v>5.407740211105375E-06</v>
+        <v>5.245715104532495E-06</v>
       </c>
       <c r="G3">
-        <v>2.741026239014889E-06</v>
+        <v>1.620555624199803E-05</v>
       </c>
       <c r="H3">
-        <v>2.741026239014889E-07</v>
+        <v>5.360229089629117E-07</v>
       </c>
       <c r="I3">
         <v>1594</v>
@@ -632,13 +632,13 @@
         <v>16904215.74193548</v>
       </c>
       <c r="M3">
-        <v>5.251944328878693E-06</v>
+        <v>1.114337410712863E-05</v>
       </c>
       <c r="N3">
-        <v>2.662057837345587E-06</v>
+        <v>1.089432380723474E-05</v>
       </c>
       <c r="O3">
-        <v>2.662057837345587E-07</v>
+        <v>1.64633488029617E-06</v>
       </c>
     </row>
     <row r="4" spans="1:15">
@@ -658,13 +658,13 @@
         <v>20904961.67247387</v>
       </c>
       <c r="F4">
-        <v>4.246838687912977E-06</v>
+        <v>4.1195961680904E-06</v>
       </c>
       <c r="G4">
-        <v>2.1525990195549E-06</v>
+        <v>1.272664375894625E-05</v>
       </c>
       <c r="H4">
-        <v>2.1525990195549E-07</v>
+        <v>4.209526971574026E-07</v>
       </c>
       <c r="I4">
         <v>2218</v>
@@ -679,13 +679,13 @@
         <v>22645091.18012422</v>
       </c>
       <c r="M4">
-        <v>3.920496468476264E-06</v>
+        <v>8.318359087259224E-06</v>
       </c>
       <c r="N4">
-        <v>1.987185639574588E-06</v>
+        <v>8.1324468307568E-06</v>
       </c>
       <c r="O4">
-        <v>1.987185639574587E-07</v>
+        <v>1.228963918874684E-06</v>
       </c>
     </row>
     <row r="5" spans="1:15">
@@ -705,13 +705,13 @@
         <v>16253029.85468957</v>
       </c>
       <c r="F5">
-        <v>5.462366143035409E-06</v>
+        <v>5.29870435050923E-06</v>
       </c>
       <c r="G5">
-        <v>2.768714535217317E-06</v>
+        <v>1.636925560210149E-05</v>
       </c>
       <c r="H5">
-        <v>2.768714535217317E-07</v>
+        <v>5.414375091091643E-07</v>
       </c>
       <c r="I5">
         <v>2221</v>
@@ -726,13 +726,13 @@
         <v>25177868.68965517</v>
       </c>
       <c r="M5">
-        <v>3.526112598898294E-06</v>
+        <v>7.481570514242755E-06</v>
       </c>
       <c r="N5">
-        <v>1.787283926001614E-06</v>
+        <v>7.314360173610159E-06</v>
       </c>
       <c r="O5">
-        <v>1.787283926001614E-07</v>
+        <v>1.105335814680553E-06</v>
       </c>
     </row>
     <row r="6" spans="1:15">
@@ -752,13 +752,13 @@
         <v>16073039.05511811</v>
       </c>
       <c r="F6">
-        <v>5.523535387150691E-06</v>
+        <v>5.358040859894317E-06</v>
       </c>
       <c r="G6">
-        <v>2.799719446066469E-06</v>
+        <v>1.655256352502187E-05</v>
       </c>
       <c r="H6">
-        <v>2.799719446066469E-07</v>
+        <v>5.475006916752206E-07</v>
       </c>
       <c r="I6">
         <v>2202</v>
@@ -773,13 +773,13 @@
         <v>21804575.42168675</v>
       </c>
       <c r="M6">
-        <v>4.071622505050007E-06</v>
+        <v>8.639012517191597E-06</v>
       </c>
       <c r="N6">
-        <v>2.063787032296129E-06</v>
+        <v>8.445933774836779E-06</v>
       </c>
       <c r="O6">
-        <v>2.063787032296129E-07</v>
+        <v>1.276337624640028E-06</v>
       </c>
     </row>
     <row r="7" spans="1:15">
@@ -799,13 +799,13 @@
         <v>4394335.285053928</v>
       </c>
       <c r="F7">
-        <v>2.020328314545313E-05</v>
+        <v>1.9597958374481E-05</v>
       </c>
       <c r="G7">
-        <v>1.024045665178408E-05</v>
+        <v>6.054385538238121E-05</v>
       </c>
       <c r="H7">
-        <v>1.024045665178408E-06</v>
+        <v>2.00257818968222E-06</v>
       </c>
       <c r="I7">
         <v>1878</v>
@@ -820,13 +820,13 @@
         <v>16596673.5483871</v>
       </c>
       <c r="M7">
-        <v>5.34926470302405E-06</v>
+        <v>1.134986474553548E-05</v>
       </c>
       <c r="N7">
-        <v>2.711386704619084E-06</v>
+        <v>1.10961994560589E-05</v>
       </c>
       <c r="O7">
-        <v>2.711386704619084E-07</v>
+        <v>1.676842044212202E-06</v>
       </c>
     </row>
     <row r="8" spans="1:15">
@@ -846,13 +846,13 @@
         <v>883998.8372093022</v>
       </c>
       <c r="F8">
-        <v>0.000100429996356409</v>
+        <v>9.742094262462202E-05</v>
       </c>
       <c r="G8">
-        <v>5.090504433474211E-05</v>
+        <v>0.0003009619343390698</v>
       </c>
       <c r="H8">
-        <v>5.090504433474211E-06</v>
+        <v>9.95476422546068E-06</v>
       </c>
       <c r="I8">
         <v>1191</v>
@@ -867,13 +867,13 @@
         <v>9021742.672811059</v>
       </c>
       <c r="M8">
-        <v>9.840670834866241E-06</v>
+        <v>2.087955806672396E-05</v>
       </c>
       <c r="N8">
-        <v>4.987949848715711E-06</v>
+        <v>2.041290764754412E-05</v>
       </c>
       <c r="O8">
-        <v>4.987949848715711E-07</v>
+        <v>3.084769873105738E-06</v>
       </c>
     </row>
     <row r="9" spans="1:15">
@@ -893,13 +893,13 @@
         <v>733821.4285714285</v>
       </c>
       <c r="F9">
-        <v>0.0001209831118898136</v>
+        <v>0.0001173582518129167</v>
       </c>
       <c r="G9">
-        <v>6.132282084975909E-05</v>
+        <v>0.0003625541441572979</v>
       </c>
       <c r="H9">
-        <v>6.132282084975909E-06</v>
+        <v>1.199201829950845E-05</v>
       </c>
       <c r="I9">
         <v>898</v>
@@ -914,13 +914,13 @@
         <v>7608744.742268042</v>
       </c>
       <c r="M9">
-        <v>1.166815329035945E-05</v>
+        <v>2.475704027151396E-05</v>
       </c>
       <c r="N9">
-        <v>5.914247556501184E-06</v>
+        <v>2.42037295556724E-05</v>
       </c>
       <c r="O9">
-        <v>5.914247556501184E-07</v>
+        <v>3.657633544387288E-06</v>
       </c>
     </row>
     <row r="10" spans="1:15">
@@ -940,13 +940,13 @@
         <v>803058.320610687</v>
       </c>
       <c r="F10">
-        <v>0.0001105523692631528</v>
+        <v>0.0001072400319998053</v>
       </c>
       <c r="G10">
-        <v>5.603578077091546E-05</v>
+        <v>0.0003312959883133791</v>
       </c>
       <c r="H10">
-        <v>5.603578077091546E-06</v>
+        <v>1.095810823964569E-05</v>
       </c>
       <c r="I10">
         <v>635</v>
@@ -961,13 +961,13 @@
         <v>4964507.015457788</v>
       </c>
       <c r="M10">
-        <v>1.788294380964096E-05</v>
+        <v>3.794334450802059E-05</v>
       </c>
       <c r="N10">
-        <v>9.064344125184088E-06</v>
+        <v>3.709532475764226E-05</v>
       </c>
       <c r="O10">
-        <v>9.064344125184088E-07</v>
+        <v>5.605793266752737E-06</v>
       </c>
     </row>
     <row r="11" spans="1:15">
@@ -987,13 +987,13 @@
         <v>237727.4215033302</v>
       </c>
       <c r="F11">
-        <v>0.0003734529211589346</v>
+        <v>0.0003622636356184665</v>
       </c>
       <c r="G11">
-        <v>0.0001892924245567927</v>
+        <v>0.001119138878962994</v>
       </c>
       <c r="H11">
-        <v>1.892924245567928E-05</v>
+        <v>3.701718524666169E-05</v>
       </c>
       <c r="I11">
         <v>561</v>
@@ -1008,13 +1008,13 @@
         <v>3775432.384851587</v>
       </c>
       <c r="M11">
-        <v>2.351518738786524E-05</v>
+        <v>4.989362298098867E-05</v>
       </c>
       <c r="N11">
-        <v>1.191916459173165E-05</v>
+        <v>4.877851891585112E-05</v>
       </c>
       <c r="O11">
-        <v>1.191916459173165E-06</v>
+        <v>7.371341124175372E-06</v>
       </c>
     </row>
     <row r="12" spans="1:15">
@@ -1034,13 +1034,13 @@
         <v>303586.2940461726</v>
       </c>
       <c r="F12">
-        <v>0.0002924374444470059</v>
+        <v>0.000283675520565174</v>
       </c>
       <c r="G12">
-        <v>0.0001482280355949005</v>
+        <v>0.0008763570860005174</v>
       </c>
       <c r="H12">
-        <v>1.482280355949005E-05</v>
+        <v>2.898681584966943E-05</v>
       </c>
       <c r="I12">
         <v>800</v>
@@ -1055,13 +1055,13 @@
         <v>5930137.542277339</v>
       </c>
       <c r="M12">
-        <v>1.497098496739183E-05</v>
+        <v>3.176486188677179E-05</v>
       </c>
       <c r="N12">
-        <v>7.588356876916338E-06</v>
+        <v>3.105492894339807E-05</v>
       </c>
       <c r="O12">
-        <v>7.588356876916339E-07</v>
+        <v>4.692977152990704E-06</v>
       </c>
     </row>
     <row r="13" spans="1:15">
@@ -1081,13 +1081,13 @@
         <v>5524490.362164466</v>
       </c>
       <c r="F13">
-        <v>1.607026063580939E-05</v>
+        <v>1.558876825812013E-05</v>
       </c>
       <c r="G13">
-        <v>8.145547742863514E-06</v>
+        <v>4.815828837752973E-05</v>
       </c>
       <c r="H13">
-        <v>8.145547742863513E-07</v>
+        <v>1.592907114159976E-06</v>
       </c>
       <c r="I13">
         <v>904</v>
@@ -1102,13 +1102,13 @@
         <v>6582321.328903655</v>
       </c>
       <c r="M13">
-        <v>1.348764297029345E-05</v>
+        <v>2.861756371158118E-05</v>
       </c>
       <c r="N13">
-        <v>6.836493958810601E-06</v>
+        <v>2.797797172121245E-05</v>
       </c>
       <c r="O13">
-        <v>6.8364939588106E-07</v>
+        <v>4.227991708304423E-06</v>
       </c>
     </row>
     <row r="14" spans="1:15">
@@ -1128,13 +1128,13 @@
         <v>7032066.728971962</v>
       </c>
       <c r="F14">
-        <v>1.262502240404351E-05</v>
+        <v>1.224675523131592E-05</v>
       </c>
       <c r="G14">
-        <v>6.399256681481844E-06</v>
+        <v>3.783382755796099E-05</v>
       </c>
       <c r="H14">
-        <v>6.399256681481843E-07</v>
+        <v>1.251410195489783E-06</v>
       </c>
       <c r="I14">
         <v>1373</v>
@@ -1149,13 +1149,13 @@
         <v>11172685.54455445</v>
       </c>
       <c r="M14">
-        <v>7.946164746690755E-06</v>
+        <v>1.685986768792676E-05</v>
       </c>
       <c r="N14">
-        <v>4.027679810780401E-06</v>
+        <v>1.64830558656293E-05</v>
       </c>
       <c r="O14">
-        <v>4.0276798107804E-07</v>
+        <v>2.49089620297819E-06</v>
       </c>
     </row>
     <row r="15" spans="1:15">
@@ -1175,13 +1175,13 @@
         <v>20244539.60988297</v>
       </c>
       <c r="F15">
-        <v>4.385380043745694E-06</v>
+        <v>4.253986588954485E-06</v>
       </c>
       <c r="G15">
-        <v>2.222821603610681E-06</v>
+        <v>1.31418152809027E-05</v>
       </c>
       <c r="H15">
-        <v>2.22282160361068E-07</v>
+        <v>4.346851135949776E-07</v>
       </c>
       <c r="I15">
         <v>2247</v>
@@ -1196,13 +1196,13 @@
         <v>36389445.51724138</v>
       </c>
       <c r="M15">
-        <v>2.439718405655175E-06</v>
+        <v>5.176500969511887E-06</v>
       </c>
       <c r="N15">
-        <v>1.236622305186786E-06</v>
+        <v>5.060808082737746E-06</v>
       </c>
       <c r="O15">
-        <v>1.236622305186786E-07</v>
+        <v>7.647821945188502E-07</v>
       </c>
     </row>
     <row r="16" spans="1:15">
@@ -1222,13 +1222,13 @@
         <v>25785786.12244898</v>
       </c>
       <c r="F16">
-        <v>3.442982097905038E-06</v>
+        <v>3.339824490556228E-06</v>
       </c>
       <c r="G16">
-        <v>1.745147492743036E-06</v>
+        <v>1.031769978765077E-05</v>
       </c>
       <c r="H16">
-        <v>1.745147492743036E-07</v>
+        <v>3.412732874697493E-07</v>
       </c>
       <c r="I16">
         <v>2065</v>
@@ -1243,13 +1243,13 @@
         <v>35730151.57894737</v>
       </c>
       <c r="M16">
-        <v>2.48473617034164E-06</v>
+        <v>5.272017936553896E-06</v>
       </c>
       <c r="N16">
-        <v>1.259440500848995E-06</v>
+        <v>5.1541902808078E-06</v>
       </c>
       <c r="O16">
-        <v>1.259440500848995E-07</v>
+        <v>7.788939808583898E-07</v>
       </c>
     </row>
     <row r="17" spans="1:15">
@@ -1269,13 +1269,13 @@
         <v>18584878.05510535</v>
       </c>
       <c r="F17">
-        <v>4.777002019424698E-06</v>
+        <v>4.633874903276132E-06</v>
       </c>
       <c r="G17">
-        <v>2.421323393490779E-06</v>
+        <v>1.431540197418271E-05</v>
       </c>
       <c r="H17">
-        <v>2.421323393490779E-07</v>
+        <v>4.735032413937525E-07</v>
       </c>
       <c r="I17">
         <v>2190</v>
@@ -1290,13 +1290,13 @@
         <v>35998344</v>
       </c>
       <c r="M17">
-        <v>2.466224557440753E-06</v>
+        <v>5.23274070607248E-06</v>
       </c>
       <c r="N17">
-        <v>1.250057502645122E-06</v>
+        <v>5.115790881936124E-06</v>
       </c>
       <c r="O17">
-        <v>1.250057502645122E-07</v>
+        <v>7.730911177469718E-07</v>
       </c>
     </row>
     <row r="18" spans="1:15">
@@ -1316,13 +1316,13 @@
         <v>14629985.82857143</v>
       </c>
       <c r="F18">
-        <v>6.068358578079982E-06</v>
+        <v>5.886540220142466E-06</v>
       </c>
       <c r="G18">
-        <v>3.075874476386564E-06</v>
+        <v>1.818525343205879E-05</v>
       </c>
       <c r="H18">
-        <v>3.075874476386565E-07</v>
+        <v>6.015043420489282E-07</v>
       </c>
       <c r="I18">
         <v>2192</v>
@@ -1337,13 +1337,13 @@
         <v>34812772.17391305</v>
       </c>
       <c r="M18">
-        <v>2.550213454891918E-06</v>
+        <v>5.410945128384665E-06</v>
       </c>
       <c r="N18">
-        <v>1.29262903210336E-06</v>
+        <v>5.290012501158995E-06</v>
       </c>
       <c r="O18">
-        <v>1.29262903210336E-07</v>
+        <v>7.994192436319223E-07</v>
       </c>
     </row>
     <row r="19" spans="1:15">
@@ -1363,13 +1363,13 @@
         <v>9053809.07348243</v>
       </c>
       <c r="F19">
-        <v>9.805817560260517E-06</v>
+        <v>9.512018566001755E-06</v>
       </c>
       <c r="G19">
-        <v>4.970283737460275E-06</v>
+        <v>2.938542196336236E-05</v>
       </c>
       <c r="H19">
-        <v>4.970283737460275E-07</v>
+        <v>9.719665975477872E-07</v>
       </c>
       <c r="I19">
         <v>1941</v>
@@ -1384,13 +1384,13 @@
         <v>31589486.73267327</v>
       </c>
       <c r="M19">
-        <v>2.810428695828543E-06</v>
+        <v>5.963059849439319E-06</v>
       </c>
       <c r="N19">
-        <v>1.42452456986128E-06</v>
+        <v>5.829787661903407E-06</v>
       </c>
       <c r="O19">
-        <v>1.42452456986128E-07</v>
+        <v>8.809893062053204E-07</v>
       </c>
     </row>
     <row r="20" spans="1:15">
@@ -1410,13 +1410,13 @@
         <v>2462427.021110242</v>
       </c>
       <c r="F20">
-        <v>3.605386037388896E-05</v>
+        <v>3.497362531425228E-05</v>
       </c>
       <c r="G20">
-        <v>1.827465326453034E-05</v>
+        <v>0.0001080438111339621</v>
       </c>
       <c r="H20">
-        <v>1.827465326453034E-06</v>
+        <v>3.573709971730377E-06</v>
       </c>
       <c r="I20">
         <v>1192</v>
@@ -1431,13 +1431,13 @@
         <v>21531449.67032967</v>
       </c>
       <c r="M20">
-        <v>4.123270906479595E-06</v>
+        <v>8.748598115043492E-06</v>
       </c>
       <c r="N20">
-        <v>2.089966104883778E-06</v>
+        <v>8.55307017500881E-06</v>
       </c>
       <c r="O20">
-        <v>2.089966104883777E-07</v>
+        <v>1.292527926642567E-06</v>
       </c>
     </row>
     <row r="21" spans="1:15">
@@ -1457,13 +1457,13 @@
         <v>1341308.16</v>
       </c>
       <c r="F21">
-        <v>6.618911496072611E-05</v>
+        <v>6.420597635072913E-05</v>
       </c>
       <c r="G21">
-        <v>3.354933738716687E-05</v>
+        <v>0.0001983511380412388</v>
       </c>
       <c r="H21">
-        <v>3.354933738716687E-06</v>
+        <v>6.560759311268189E-06</v>
       </c>
       <c r="I21">
         <v>888</v>
@@ -1478,13 +1478,13 @@
         <v>19462118.4</v>
       </c>
       <c r="M21">
-        <v>4.561682247293286E-06</v>
+        <v>9.678802488427981E-06</v>
       </c>
       <c r="N21">
-        <v>2.312184063169609E-06</v>
+        <v>9.462484823851447E-06</v>
       </c>
       <c r="O21">
-        <v>2.312184063169609E-07</v>
+        <v>1.429957388400227E-06</v>
       </c>
     </row>
     <row r="22" spans="1:15">
@@ -1504,13 +1504,13 @@
         <v>998576.0946745563</v>
       </c>
       <c r="F22">
-        <v>8.890659457348025E-05</v>
+        <v>8.624280158445729E-05</v>
       </c>
       <c r="G22">
-        <v>4.50641671075311E-05</v>
+        <v>0.0002664293701990811</v>
       </c>
       <c r="H22">
-        <v>4.50641671075311E-06</v>
+        <v>8.812548234361638E-06</v>
       </c>
       <c r="I22">
         <v>744</v>
@@ -1525,13 +1525,13 @@
         <v>15749612.87830006</v>
       </c>
       <c r="M22">
-        <v>5.636963948639128E-06</v>
+        <v>1.196029397392603E-05</v>
       </c>
       <c r="N22">
-        <v>2.857213085027718E-06</v>
+        <v>1.169298581641566E-05</v>
       </c>
       <c r="O22">
-        <v>2.857213085027718E-07</v>
+        <v>1.767027559029364E-06</v>
       </c>
     </row>
     <row r="23" spans="1:15">
@@ -1551,13 +1551,13 @@
         <v>949038.7924528302</v>
       </c>
       <c r="F23">
-        <v>9.354728247782622E-05</v>
+        <v>9.074444657569718E-05</v>
       </c>
       <c r="G23">
-        <v>4.741639684052918E-05</v>
+        <v>0.0002803362750982842</v>
       </c>
       <c r="H23">
-        <v>4.741639684052918E-06</v>
+        <v>9.272539826592373E-06</v>
       </c>
       <c r="I23">
         <v>709</v>
@@ -1572,13 +1572,13 @@
         <v>74230945.22292994</v>
       </c>
       <c r="M23">
-        <v>1.19599716443562E-06</v>
+        <v>2.5376209266134E-06</v>
       </c>
       <c r="N23">
-        <v>6.062161793151935E-07</v>
+        <v>2.480906035170801E-06</v>
       </c>
       <c r="O23">
-        <v>6.062161793151935E-08</v>
+        <v>3.749110282298186E-07</v>
       </c>
     </row>
     <row r="24" spans="1:15">
@@ -1598,13 +1598,13 @@
         <v>1094639.737130339</v>
       </c>
       <c r="F24">
-        <v>8.110430947148132E-05</v>
+        <v>7.867428623207897E-05</v>
       </c>
       <c r="G24">
-        <v>4.110941570417503E-05</v>
+        <v>0.0002430480010687948</v>
       </c>
       <c r="H24">
-        <v>4.110941570417502E-06</v>
+        <v>8.039174626594228E-06</v>
       </c>
       <c r="I24">
         <v>800</v>
@@ -1619,13 +1619,13 @@
         <v>16234666.66666667</v>
       </c>
       <c r="M24">
-        <v>5.46854467805519E-06</v>
+        <v>1.160294842312746E-05</v>
       </c>
       <c r="N24">
-        <v>2.771846254927727E-06</v>
+        <v>1.134362680683311E-05</v>
       </c>
       <c r="O24">
-        <v>2.771846254927726E-07</v>
+        <v>1.714232917214192E-06</v>
       </c>
     </row>
     <row r="25" spans="1:15">
@@ -1645,13 +1645,13 @@
         <v>5524169.676025919</v>
       </c>
       <c r="F25">
-        <v>1.607119353797044E-05</v>
+        <v>1.558967320894362E-05</v>
       </c>
       <c r="G25">
-        <v>8.146020603837236E-06</v>
+        <v>4.816108403668659E-05</v>
       </c>
       <c r="H25">
-        <v>8.146020603837237E-07</v>
+        <v>1.592999584750393E-06</v>
       </c>
       <c r="I25">
         <v>910</v>
@@ -1666,13 +1666,13 @@
         <v>125699294.1176471</v>
       </c>
       <c r="M25">
-        <v>7.062887713347635E-07</v>
+        <v>1.498576434515988E-06</v>
       </c>
       <c r="N25">
-        <v>3.57997237103676E-07</v>
+        <v>1.465083804111399E-06</v>
       </c>
       <c r="O25">
-        <v>3.57997237103676E-08</v>
+        <v>2.21401402413229E-07</v>
       </c>
     </row>
     <row r="26" spans="1:15">
@@ -1692,13 +1692,13 @@
         <v>18246291.95039459</v>
       </c>
       <c r="F26">
-        <v>4.865646140123285E-06</v>
+        <v>4.719863095150004E-06</v>
       </c>
       <c r="G26">
-        <v>2.466254520224688E-06</v>
+        <v>1.458104478012841E-05</v>
       </c>
       <c r="H26">
-        <v>2.466254520224689E-07</v>
+        <v>4.822897728439391E-07</v>
       </c>
       <c r="I26">
         <v>1097</v>
@@ -1713,13 +1713,13 @@
         <v>196000513.0434783</v>
       </c>
       <c r="M26">
-        <v>4.529579980247611E-07</v>
+        <v>9.610689129074597E-07</v>
       </c>
       <c r="N26">
-        <v>2.29591235763846E-07</v>
+        <v>9.395893772948864E-07</v>
       </c>
       <c r="O26">
-        <v>2.295912357638461E-08</v>
+        <v>1.419894242512852E-07</v>
       </c>
     </row>
     <row r="27" spans="1:15">
@@ -1739,13 +1739,13 @@
         <v>30569221.17340287</v>
       </c>
       <c r="F27">
-        <v>2.904228390262168E-06</v>
+        <v>2.817212761538386E-06</v>
       </c>
       <c r="G27">
-        <v>1.472068906981275E-06</v>
+        <v>8.70319850449707E-06</v>
       </c>
       <c r="H27">
-        <v>1.472068906981275E-07</v>
+        <v>2.878712529207826E-07</v>
       </c>
       <c r="I27">
         <v>1672</v>
@@ -1760,13 +1760,13 @@
         <v>61074816</v>
       </c>
       <c r="M27">
-        <v>1.453626974496329E-06</v>
+        <v>3.084249979566046E-06</v>
       </c>
       <c r="N27">
-        <v>7.36801237354526E-07</v>
+        <v>3.015318130471322E-06</v>
       </c>
       <c r="O27">
-        <v>7.36801237354526E-08</v>
+        <v>4.55670631901699E-07</v>
       </c>
     </row>
     <row r="28" spans="1:15">

</xml_diff>